<commit_message>
Re-run notebook and dashboard with verified live UN Comtrade API data
- Confirmed API key active: real bilateral trade stats (Canada reporter 124)
- Fetched 135,222 world records + 43,173 China records (2021-2024)
- Canada total imports: USD 8,650B across 102 HS2 chapters
- China share: 15.3% overall; Yiwu universe gap = USD 881.6B
- Regenerated all 9 figures from live data (no demo/synthetic data)
- Re-exported HTML report and Excel workbook
- Streamlit dashboard running on port 8501 with live cached data

https://claude.ai/code/session_01P1T4h6yXr97FBHTbptyQHn
</commit_message>
<xml_diff>
--- a/canada-gap/yiwu_canada_opportunity.xlsx
+++ b/canada-gap/yiwu_canada_opportunity.xlsx
@@ -486,7 +486,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Plastics</t>
+          <t>Plastics and articles thereof</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -495,19 +495,19 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>62.208</v>
+        <v>324.911</v>
       </c>
       <c r="F2" t="n">
-        <v>12.247</v>
+        <v>49.38</v>
       </c>
       <c r="G2" t="n">
-        <v>49.961</v>
+        <v>275.531</v>
       </c>
       <c r="H2" t="n">
-        <v>19.69</v>
+        <v>15.2</v>
       </c>
       <c r="I2" t="n">
-        <v>40.1234</v>
+        <v>233.6504</v>
       </c>
     </row>
     <row r="3">
@@ -521,7 +521,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Articles of iron or steel</t>
+          <t>Iron or steel articles</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -530,19 +530,19 @@
         </is>
       </c>
       <c r="E3" t="n">
-        <v>31.764</v>
+        <v>198.18</v>
       </c>
       <c r="F3" t="n">
-        <v>8.536</v>
+        <v>45.706</v>
       </c>
       <c r="G3" t="n">
-        <v>23.227</v>
+        <v>152.474</v>
       </c>
       <c r="H3" t="n">
-        <v>26.87</v>
+        <v>23.06</v>
       </c>
       <c r="I3" t="n">
-        <v>16.9862</v>
+        <v>117.3132</v>
       </c>
     </row>
     <row r="4">
@@ -556,7 +556,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Furniture, bedding, lighting</t>
+          <t>Furniture; bedding, mattresses, mattress supports, cushions and similar stuffed furnishings; lamps and lighting fittings, n.e.c.; illuminated signs, illuminated name-plates and the like; prefabricated buildings</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -565,19 +565,19 @@
         </is>
       </c>
       <c r="E4" t="n">
-        <v>32.926</v>
+        <v>157.122</v>
       </c>
       <c r="F4" t="n">
-        <v>16.708</v>
+        <v>62.013</v>
       </c>
       <c r="G4" t="n">
-        <v>16.218</v>
+        <v>95.10899999999999</v>
       </c>
       <c r="H4" t="n">
-        <v>50.74</v>
+        <v>39.47</v>
       </c>
       <c r="I4" t="n">
-        <v>7.9892</v>
+        <v>57.5695</v>
       </c>
     </row>
     <row r="5">
@@ -586,12 +586,12 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>62</t>
+          <t>61</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Woven apparel</t>
+          <t>Apparel and clothing accessories; knitted or crocheted</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -600,19 +600,19 @@
         </is>
       </c>
       <c r="E5" t="n">
-        <v>19.115</v>
+        <v>97.56399999999999</v>
       </c>
       <c r="F5" t="n">
-        <v>8.170999999999999</v>
+        <v>29.303</v>
       </c>
       <c r="G5" t="n">
-        <v>10.944</v>
+        <v>68.261</v>
       </c>
       <c r="H5" t="n">
-        <v>42.75</v>
+        <v>30.03</v>
       </c>
       <c r="I5" t="n">
-        <v>6.2655</v>
+        <v>47.7623</v>
       </c>
     </row>
     <row r="6">
@@ -621,12 +621,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>62</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Knitted apparel</t>
+          <t>Apparel and clothing accessories; not knitted or crocheted</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -635,19 +635,19 @@
         </is>
       </c>
       <c r="E6" t="n">
-        <v>23.506</v>
+        <v>76.456</v>
       </c>
       <c r="F6" t="n">
-        <v>12.624</v>
+        <v>23.399</v>
       </c>
       <c r="G6" t="n">
-        <v>10.882</v>
+        <v>53.057</v>
       </c>
       <c r="H6" t="n">
-        <v>53.71</v>
+        <v>30.6</v>
       </c>
       <c r="I6" t="n">
-        <v>5.0371</v>
+        <v>36.8216</v>
       </c>
     </row>
     <row r="7">
@@ -661,7 +661,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Glass</t>
+          <t>Glass and glassware</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -670,19 +670,19 @@
         </is>
       </c>
       <c r="E7" t="n">
-        <v>7.838</v>
+        <v>43.033</v>
       </c>
       <c r="F7" t="n">
-        <v>2.141</v>
+        <v>9.353999999999999</v>
       </c>
       <c r="G7" t="n">
-        <v>5.696</v>
+        <v>33.679</v>
       </c>
       <c r="H7" t="n">
-        <v>27.32</v>
+        <v>21.74</v>
       </c>
       <c r="I7" t="n">
-        <v>4.14</v>
+        <v>26.3568</v>
       </c>
     </row>
     <row r="8">
@@ -691,33 +691,33 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>95</t>
+          <t>83</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Toys, games, sports</t>
+          <t>Metal; miscellaneous products of base metal</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Toys, Games &amp; Sports</t>
+          <t>Home Décor &amp; Hardware</t>
         </is>
       </c>
       <c r="E8" t="n">
-        <v>12.288</v>
+        <v>47.36</v>
       </c>
       <c r="F8" t="n">
-        <v>6.12</v>
+        <v>12.771</v>
       </c>
       <c r="G8" t="n">
-        <v>6.167</v>
+        <v>34.589</v>
       </c>
       <c r="H8" t="n">
-        <v>49.81</v>
+        <v>26.97</v>
       </c>
       <c r="I8" t="n">
-        <v>3.0954</v>
+        <v>25.2603</v>
       </c>
     </row>
     <row r="9">
@@ -726,33 +726,33 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>82</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Footwear</t>
+          <t>Tools, implements, cutlery, spoons and forks, of base metal; parts thereof, of base metal</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Textiles &amp; Apparel</t>
+          <t>Kitchenware &amp; Tableware</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>17.778</v>
+        <v>37.909</v>
       </c>
       <c r="F9" t="n">
-        <v>10.858</v>
+        <v>11.076</v>
       </c>
       <c r="G9" t="n">
-        <v>6.92</v>
+        <v>26.833</v>
       </c>
       <c r="H9" t="n">
-        <v>61.08</v>
+        <v>29.22</v>
       </c>
       <c r="I9" t="n">
-        <v>2.6931</v>
+        <v>18.9923</v>
       </c>
     </row>
     <row r="10">
@@ -761,33 +761,33 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>42</t>
+          <t>64</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Articles of leather</t>
+          <t>Footwear; gaiters and the like; parts of such articles</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Bags &amp; Travel Goods</t>
+          <t>Textiles &amp; Apparel</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>10.725</v>
+        <v>41.393</v>
       </c>
       <c r="F10" t="n">
-        <v>5.541</v>
+        <v>13.915</v>
       </c>
       <c r="G10" t="n">
-        <v>5.184</v>
+        <v>27.478</v>
       </c>
       <c r="H10" t="n">
-        <v>51.67</v>
+        <v>33.62</v>
       </c>
       <c r="I10" t="n">
-        <v>2.5053</v>
+        <v>18.24</v>
       </c>
     </row>
     <row r="11">
@@ -796,33 +796,33 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>69</t>
+          <t>95</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Ceramic products</t>
+          <t>Toys, games and sports requisites; parts and accessories thereof</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Kitchenware &amp; Tableware</t>
+          <t>Toys, Games &amp; Sports</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>5.85</v>
+        <v>85.108</v>
       </c>
       <c r="F11" t="n">
-        <v>2.338</v>
+        <v>50.864</v>
       </c>
       <c r="G11" t="n">
-        <v>3.512</v>
+        <v>34.244</v>
       </c>
       <c r="H11" t="n">
-        <v>39.97</v>
+        <v>59.76</v>
       </c>
       <c r="I11" t="n">
-        <v>2.108</v>
+        <v>13.7799</v>
       </c>
     </row>
     <row r="12">
@@ -831,33 +831,33 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>42</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Carpets</t>
+          <t>Articles of leather; saddlery and harness; travel goods, handbags and similar containers; articles of animal gut (other than silk-worm gut)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Textiles &amp; Apparel</t>
+          <t>Bags &amp; Travel Goods</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>3.452</v>
+        <v>32.022</v>
       </c>
       <c r="F12" t="n">
-        <v>1.199</v>
+        <v>12.474</v>
       </c>
       <c r="G12" t="n">
-        <v>2.252</v>
+        <v>19.548</v>
       </c>
       <c r="H12" t="n">
-        <v>34.74</v>
+        <v>38.95</v>
       </c>
       <c r="I12" t="n">
-        <v>1.4699</v>
+        <v>11.9339</v>
       </c>
     </row>
     <row r="13">
@@ -880,19 +880,19 @@
         </is>
       </c>
       <c r="E13" t="n">
-        <v>7.657</v>
+        <v>27.322</v>
       </c>
       <c r="F13" t="n">
-        <v>4.326</v>
+        <v>9.807</v>
       </c>
       <c r="G13" t="n">
-        <v>3.331</v>
+        <v>17.516</v>
       </c>
       <c r="H13" t="n">
-        <v>56.5</v>
+        <v>35.89</v>
       </c>
       <c r="I13" t="n">
-        <v>1.449</v>
+        <v>11.2293</v>
       </c>
     </row>
     <row r="14">
@@ -901,12 +901,12 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>63</t>
+          <t>57</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Other made-up textiles</t>
+          <t>Carpets and other textile floor coverings</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -915,19 +915,19 @@
         </is>
       </c>
       <c r="E14" t="n">
-        <v>5.822</v>
+        <v>11.302</v>
       </c>
       <c r="F14" t="n">
-        <v>3.04</v>
+        <v>1.321</v>
       </c>
       <c r="G14" t="n">
-        <v>2.782</v>
+        <v>9.98</v>
       </c>
       <c r="H14" t="n">
-        <v>52.22</v>
+        <v>11.69</v>
       </c>
       <c r="I14" t="n">
-        <v>1.3292</v>
+        <v>8.813599999999999</v>
       </c>
     </row>
     <row r="15">
@@ -936,33 +936,33 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>63</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Misc articles of base metal</t>
+          <t>Textiles, made up articles; sets; worn clothing and worn textile articles; rags</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Home Décor &amp; Hardware</t>
+          <t>Textiles &amp; Apparel</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>7.679</v>
+        <v>29.4</v>
       </c>
       <c r="F15" t="n">
-        <v>4.658</v>
+        <v>13.5</v>
       </c>
       <c r="G15" t="n">
-        <v>3.02</v>
+        <v>15.9</v>
       </c>
       <c r="H15" t="n">
-        <v>60.66</v>
+        <v>45.92</v>
       </c>
       <c r="I15" t="n">
-        <v>1.1883</v>
+        <v>8.598800000000001</v>
       </c>
     </row>
     <row r="16">
@@ -971,12 +971,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>82</t>
+          <t>69</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Tools, cutlery</t>
+          <t>Ceramic products</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -985,19 +985,19 @@
         </is>
       </c>
       <c r="E16" t="n">
-        <v>9.612</v>
+        <v>19.992</v>
       </c>
       <c r="F16" t="n">
-        <v>6.257</v>
+        <v>6.971</v>
       </c>
       <c r="G16" t="n">
-        <v>3.355</v>
+        <v>13.021</v>
       </c>
       <c r="H16" t="n">
-        <v>65.09</v>
+        <v>34.87</v>
       </c>
       <c r="I16" t="n">
-        <v>1.1713</v>
+        <v>8.480700000000001</v>
       </c>
     </row>
     <row r="17">
@@ -1011,7 +1011,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Headgear</t>
+          <t>Headgear and parts thereof</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1020,19 +1020,19 @@
         </is>
       </c>
       <c r="E17" t="n">
-        <v>2.341</v>
+        <v>7.208</v>
       </c>
       <c r="F17" t="n">
-        <v>1.395</v>
+        <v>3.945</v>
       </c>
       <c r="G17" t="n">
-        <v>0.946</v>
+        <v>3.263</v>
       </c>
       <c r="H17" t="n">
-        <v>59.61</v>
+        <v>54.73</v>
       </c>
       <c r="I17" t="n">
-        <v>0.3819</v>
+        <v>1.477</v>
       </c>
     </row>
     <row r="18">
@@ -1041,33 +1041,33 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>46</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Umbrellas</t>
+          <t>Manufactures of straw, esparto or other plaiting materials; basketware and wickerwork</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Textiles &amp; Apparel</t>
+          <t>Seasonal &amp; Festive Goods</t>
         </is>
       </c>
       <c r="E18" t="n">
-        <v>0.8</v>
+        <v>0.768</v>
       </c>
       <c r="F18" t="n">
-        <v>0.396</v>
+        <v>0.362</v>
       </c>
       <c r="G18" t="n">
-        <v>0.404</v>
+        <v>0.406</v>
       </c>
       <c r="H18" t="n">
-        <v>49.47</v>
+        <v>47.09</v>
       </c>
       <c r="I18" t="n">
-        <v>0.2042</v>
+        <v>0.2149</v>
       </c>
     </row>
     <row r="19">
@@ -1076,12 +1076,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>46</t>
+          <t>67</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Basketware</t>
+          <t>Feathers and down, prepared; and articles made of feather or of down; artificial flowers; articles of human hair</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -1090,19 +1090,19 @@
         </is>
       </c>
       <c r="E19" t="n">
-        <v>1.172</v>
+        <v>2.11</v>
       </c>
       <c r="F19" t="n">
-        <v>0.708</v>
+        <v>1.631</v>
       </c>
       <c r="G19" t="n">
-        <v>0.464</v>
+        <v>0.479</v>
       </c>
       <c r="H19" t="n">
-        <v>60.44</v>
+        <v>77.3</v>
       </c>
       <c r="I19" t="n">
-        <v>0.1834</v>
+        <v>0.1087</v>
       </c>
     </row>
     <row r="20">
@@ -1111,33 +1111,33 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>66</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Feathers and artificial flowers</t>
+          <t>Umbrellas, sun umbrellas, walking-sticks, seat sticks, whips, riding crops; and parts thereof</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Seasonal &amp; Festive Goods</t>
+          <t>Textiles &amp; Apparel</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>0.392</v>
+        <v>1.471</v>
       </c>
       <c r="F20" t="n">
-        <v>0.234</v>
+        <v>1.285</v>
       </c>
       <c r="G20" t="n">
-        <v>0.159</v>
+        <v>0.186</v>
       </c>
       <c r="H20" t="n">
-        <v>59.56</v>
+        <v>87.39</v>
       </c>
       <c r="I20" t="n">
-        <v>0.06419999999999999</v>
+        <v>0.0234</v>
       </c>
     </row>
   </sheetData>

</xml_diff>